<commit_message>
mma seagrass graphs to match jumby additions
</commit_message>
<xml_diff>
--- a/mma/data/mma_seagrass.xlsx
+++ b/mma/data/mma_seagrass.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="quadrants" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="quadrats" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="site description" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="inverts" sheetId="3" r:id="rId6"/>
     <sheet state="visible" name="lookups" sheetId="4" r:id="rId7"/>
@@ -44,7 +44,7 @@
     <t>transect</t>
   </si>
   <si>
-    <t>quadrant</t>
+    <t>quadrat</t>
   </si>
   <si>
     <t>code</t>
@@ -350,6 +350,9 @@
     <t>Halophila stipulacea</t>
   </si>
   <si>
+    <t>Invasive seagrass</t>
+  </si>
+  <si>
     <t>HAL</t>
   </si>
   <si>
@@ -455,7 +458,7 @@
     <t>Sponge</t>
   </si>
   <si>
-    <t>Sponges, tunicates &amp; soft coral</t>
+    <t>Sponges, tunicates &amp; corals</t>
   </si>
   <si>
     <t>GOR</t>
@@ -468,9 +471,6 @@
   </si>
   <si>
     <t>Porites divaricata</t>
-  </si>
-  <si>
-    <t>Stony coral</t>
   </si>
   <si>
     <t>PPOR</t>
@@ -509,6 +509,18 @@
     <t>Manicina areolata</t>
   </si>
   <si>
+    <t>CARB</t>
+  </si>
+  <si>
+    <t>Cladocora arbuscula</t>
+  </si>
+  <si>
+    <t>TUN</t>
+  </si>
+  <si>
+    <t>Tunicate</t>
+  </si>
+  <si>
     <t>ANE</t>
   </si>
   <si>
@@ -540,18 +552,6 @@
   </si>
   <si>
     <t>Macrodactyla doreensis</t>
-  </si>
-  <si>
-    <t>CARB</t>
-  </si>
-  <si>
-    <t>Cladocora arbuscula</t>
-  </si>
-  <si>
-    <t>TUN</t>
-  </si>
-  <si>
-    <t>Tunicate</t>
   </si>
   <si>
     <t>CYAN</t>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="I75" s="6" t="str">
         <f>VLOOKUP(F75,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="76">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="I77" s="6" t="str">
         <f>VLOOKUP(F77,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="78">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="I79" s="6" t="str">
         <f>VLOOKUP(F79,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="80">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="I81" s="6" t="str">
         <f>VLOOKUP(F81,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="82">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="I83" s="6" t="str">
         <f>VLOOKUP(F83,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="84">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="I85" s="6" t="str">
         <f>VLOOKUP(F85,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="86">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="I87" s="6" t="str">
         <f>VLOOKUP(F87,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="88">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="I90" s="6" t="str">
         <f>VLOOKUP(F90,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="91">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="I93" s="6" t="str">
         <f>VLOOKUP(F93,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="94">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="I97" s="6" t="str">
         <f>VLOOKUP(F97,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="98">
@@ -4042,7 +4042,7 @@
       </c>
       <c r="I100" s="6" t="str">
         <f>VLOOKUP(F100,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="101">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="I102" s="6" t="str">
         <f>VLOOKUP(F102,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="103">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="I104" s="6" t="str">
         <f>VLOOKUP(F104,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="105">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="I106" s="6" t="str">
         <f>VLOOKUP(F106,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="107">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="I108" s="6" t="str">
         <f>VLOOKUP(F108,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="109">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="I110" s="6" t="str">
         <f>VLOOKUP(F110,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="111">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="I112" s="6" t="str">
         <f>VLOOKUP(F112,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="113">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="I114" s="6" t="str">
         <f>VLOOKUP(F114,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="115">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="I116" s="6" t="str">
         <f>VLOOKUP(F116,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="117">
@@ -4600,7 +4600,7 @@
       </c>
       <c r="I118" s="6" t="str">
         <f>VLOOKUP(F118,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="119">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="I133" s="6" t="str">
         <f>VLOOKUP(F133,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="134">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="I173" s="6" t="str">
         <f>VLOOKUP(F173,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="174">
@@ -13497,7 +13497,7 @@
       </c>
       <c r="I405" s="6" t="str">
         <f>VLOOKUP(F405,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="406">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="I409" s="6" t="str">
         <f>VLOOKUP(F409,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="410">
@@ -13807,7 +13807,7 @@
       </c>
       <c r="I415" s="6" t="str">
         <f>VLOOKUP(F415,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="416">
@@ -13993,7 +13993,7 @@
       </c>
       <c r="I421" s="6" t="str">
         <f>VLOOKUP(F421,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="422">
@@ -14458,7 +14458,7 @@
       </c>
       <c r="I436" s="6" t="str">
         <f>VLOOKUP(F436,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="437">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="I441" s="6" t="str">
         <f>VLOOKUP(F441,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="442">
@@ -14644,7 +14644,7 @@
       </c>
       <c r="I442" s="6" t="str">
         <f>VLOOKUP(F442,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="443">
@@ -15140,7 +15140,7 @@
       </c>
       <c r="I458" s="6" t="str">
         <f>VLOOKUP(F458,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="459">
@@ -15233,7 +15233,7 @@
       </c>
       <c r="I461" s="6" t="str">
         <f>VLOOKUP(F461,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="462">
@@ -15264,7 +15264,7 @@
       </c>
       <c r="I462" s="6" t="str">
         <f>VLOOKUP(F462,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="463">
@@ -15481,7 +15481,7 @@
       </c>
       <c r="I469" s="6" t="str">
         <f>VLOOKUP(F469,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="470">
@@ -15729,7 +15729,7 @@
       </c>
       <c r="I477" s="6" t="str">
         <f>VLOOKUP(F477,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="478">
@@ -15791,7 +15791,7 @@
       </c>
       <c r="I479" s="6" t="str">
         <f>VLOOKUP(F479,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="480">
@@ -16318,7 +16318,7 @@
       </c>
       <c r="I496" s="6" t="str">
         <f>VLOOKUP(F496,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="497">
@@ -16535,7 +16535,7 @@
       </c>
       <c r="I503" s="6" t="str">
         <f>VLOOKUP(F503,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="504">
@@ -16814,7 +16814,7 @@
       </c>
       <c r="I512" s="6" t="str">
         <f>VLOOKUP(F512,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="513">
@@ -16938,7 +16938,7 @@
       </c>
       <c r="I516" s="6" t="str">
         <f>VLOOKUP(F516,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="517">
@@ -17155,7 +17155,7 @@
       </c>
       <c r="I523" s="6" t="str">
         <f>VLOOKUP(F523,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="524">
@@ -17372,7 +17372,7 @@
       </c>
       <c r="I530" s="6" t="str">
         <f>VLOOKUP(F530,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="531">
@@ -17434,7 +17434,7 @@
       </c>
       <c r="I532" s="6" t="str">
         <f>VLOOKUP(F532,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="533">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="I534" s="6" t="str">
         <f>VLOOKUP(F534,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="535">
@@ -17558,7 +17558,7 @@
       </c>
       <c r="I536" s="6" t="str">
         <f>VLOOKUP(F536,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="537">
@@ -17713,7 +17713,7 @@
       </c>
       <c r="I541" s="6" t="str">
         <f>VLOOKUP(F541,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="542">
@@ -17868,7 +17868,7 @@
       </c>
       <c r="I546" s="6" t="str">
         <f>VLOOKUP(F546,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="547">
@@ -17930,7 +17930,7 @@
       </c>
       <c r="I548" s="6" t="str">
         <f>VLOOKUP(F548,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="549">
@@ -17961,7 +17961,7 @@
       </c>
       <c r="I549" s="6" t="str">
         <f>VLOOKUP(F549,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="550">
@@ -18116,7 +18116,7 @@
       </c>
       <c r="I554" s="6" t="str">
         <f>VLOOKUP(F554,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="555">
@@ -18271,7 +18271,7 @@
       </c>
       <c r="I559" s="6" t="str">
         <f>VLOOKUP(F559,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="560">
@@ -18302,7 +18302,7 @@
       </c>
       <c r="I560" s="6" t="str">
         <f>VLOOKUP(F560,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="561">
@@ -18488,7 +18488,7 @@
       </c>
       <c r="I566" s="6" t="str">
         <f>VLOOKUP(F566,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="567">
@@ -18550,7 +18550,7 @@
       </c>
       <c r="I568" s="6" t="str">
         <f>VLOOKUP(F568,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="569">
@@ -18674,7 +18674,7 @@
       </c>
       <c r="I572" s="6" t="str">
         <f>VLOOKUP(F572,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="573">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="I576" s="6" t="str">
         <f>VLOOKUP(F576,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="577">
@@ -18829,7 +18829,7 @@
       </c>
       <c r="I577" s="6" t="str">
         <f>VLOOKUP(F577,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="578">
@@ -18860,7 +18860,7 @@
       </c>
       <c r="I578" s="6" t="str">
         <f>VLOOKUP(F578,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="579">
@@ -19077,7 +19077,7 @@
       </c>
       <c r="I585" s="6" t="str">
         <f>VLOOKUP(F585,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="586">
@@ -19170,7 +19170,7 @@
       </c>
       <c r="I588" s="6" t="str">
         <f>VLOOKUP(F588,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="589">
@@ -19356,7 +19356,7 @@
       </c>
       <c r="I594" s="6" t="str">
         <f>VLOOKUP(F594,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="595">
@@ -19604,7 +19604,7 @@
       </c>
       <c r="I602" s="6" t="str">
         <f>VLOOKUP(F602,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="603">
@@ -19666,7 +19666,7 @@
       </c>
       <c r="I604" s="6" t="str">
         <f>VLOOKUP(F604,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="605">
@@ -19759,7 +19759,7 @@
       </c>
       <c r="I607" s="6" t="str">
         <f>VLOOKUP(F607,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="608">
@@ -19852,7 +19852,7 @@
       </c>
       <c r="I610" s="6" t="str">
         <f>VLOOKUP(F610,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="611">
@@ -23045,7 +23045,7 @@
       </c>
       <c r="I713" s="6" t="str">
         <f>VLOOKUP(F713,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="714">
@@ -23076,7 +23076,7 @@
       </c>
       <c r="I714" s="6" t="str">
         <f>VLOOKUP(F714,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="715">
@@ -23572,7 +23572,7 @@
       </c>
       <c r="I730" s="6" t="str">
         <f>VLOOKUP(F730,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="731">
@@ -23913,7 +23913,7 @@
       </c>
       <c r="I741" s="6" t="str">
         <f>VLOOKUP(F741,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="742">
@@ -24533,7 +24533,7 @@
       </c>
       <c r="I761" s="6" t="str">
         <f>VLOOKUP(F761,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="762">
@@ -24967,7 +24967,7 @@
       </c>
       <c r="I775" s="6" t="str">
         <f>VLOOKUP(F775,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="776">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="I801" s="6" t="str">
         <f>VLOOKUP(F801,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="802">
@@ -26331,7 +26331,7 @@
       </c>
       <c r="I819" s="6" t="str">
         <f>VLOOKUP(F819,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="820">
@@ -26796,7 +26796,7 @@
       </c>
       <c r="I834" s="6" t="str">
         <f>VLOOKUP(F834,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="835">
@@ -26951,7 +26951,7 @@
       </c>
       <c r="I839" s="6" t="str">
         <f>VLOOKUP(F839,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="840">
@@ -27447,7 +27447,7 @@
       </c>
       <c r="I855" s="6" t="str">
         <f>VLOOKUP(F855,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="856">
@@ -28966,7 +28966,7 @@
       </c>
       <c r="I904" s="6" t="str">
         <f>VLOOKUP(F904,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="905">
@@ -29586,7 +29586,7 @@
       </c>
       <c r="I924" s="6" t="str">
         <f>VLOOKUP(F924,lookups!$2:$110,3,FALSE)</f>
-        <v>Stony coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="925">
@@ -31198,7 +31198,7 @@
       </c>
       <c r="I976" s="6" t="str">
         <f>VLOOKUP(F976,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="977">
@@ -31787,7 +31787,7 @@
       </c>
       <c r="I995" s="6" t="str">
         <f>VLOOKUP(F995,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="996">
@@ -33461,7 +33461,7 @@
       </c>
       <c r="I1049" s="6" t="str">
         <f>VLOOKUP(F1049,lookups!$2:$110,3,FALSE)</f>
-        <v>Sponges, tunicates &amp; soft coral</v>
+        <v>Sponges, tunicates &amp; corals</v>
       </c>
     </row>
     <row r="1050">
@@ -33988,7 +33988,7 @@
       </c>
       <c r="I1066" s="6" t="str">
         <f>VLOOKUP(F1066,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1067">
@@ -34112,7 +34112,7 @@
       </c>
       <c r="I1070" s="6" t="str">
         <f>VLOOKUP(F1070,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1071">
@@ -34236,7 +34236,7 @@
       </c>
       <c r="I1074" s="6" t="str">
         <f>VLOOKUP(F1074,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1075">
@@ -34360,7 +34360,7 @@
       </c>
       <c r="I1078" s="6" t="str">
         <f>VLOOKUP(F1078,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1079">
@@ -34546,7 +34546,7 @@
       </c>
       <c r="I1084" s="6" t="str">
         <f>VLOOKUP(F1084,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1085">
@@ -34639,7 +34639,7 @@
       </c>
       <c r="I1087" s="6" t="str">
         <f>VLOOKUP(F1087,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1088">
@@ -34763,7 +34763,7 @@
       </c>
       <c r="I1091" s="6" t="str">
         <f>VLOOKUP(F1091,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1092">
@@ -34887,7 +34887,7 @@
       </c>
       <c r="I1095" s="6" t="str">
         <f>VLOOKUP(F1095,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1096">
@@ -34980,7 +34980,7 @@
       </c>
       <c r="I1098" s="6" t="str">
         <f>VLOOKUP(F1098,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1099">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="I1101" s="6" t="str">
         <f>VLOOKUP(F1101,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1102">
@@ -35228,7 +35228,7 @@
       </c>
       <c r="I1106" s="6" t="str">
         <f>VLOOKUP(F1106,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1107">
@@ -35290,7 +35290,7 @@
       </c>
       <c r="I1108" s="6" t="str">
         <f>VLOOKUP(F1108,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1109">
@@ -35383,7 +35383,7 @@
       </c>
       <c r="I1111" s="6" t="str">
         <f>VLOOKUP(F1111,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1112">
@@ -35538,7 +35538,7 @@
       </c>
       <c r="I1116" s="6" t="str">
         <f>VLOOKUP(F1116,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1117">
@@ -35662,7 +35662,7 @@
       </c>
       <c r="I1120" s="6" t="str">
         <f>VLOOKUP(F1120,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1121">
@@ -35817,7 +35817,7 @@
       </c>
       <c r="I1125" s="6" t="str">
         <f>VLOOKUP(F1125,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1126">
@@ -35910,7 +35910,7 @@
       </c>
       <c r="I1128" s="6" t="str">
         <f>VLOOKUP(F1128,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1129">
@@ -36034,7 +36034,7 @@
       </c>
       <c r="I1132" s="6" t="str">
         <f>VLOOKUP(F1132,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1133">
@@ -36189,7 +36189,7 @@
       </c>
       <c r="I1137" s="6" t="str">
         <f>VLOOKUP(F1137,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1138">
@@ -36344,7 +36344,7 @@
       </c>
       <c r="I1142" s="6" t="str">
         <f>VLOOKUP(F1142,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1143">
@@ -36406,7 +36406,7 @@
       </c>
       <c r="I1144" s="6" t="str">
         <f>VLOOKUP(F1144,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1145">
@@ -36468,7 +36468,7 @@
       </c>
       <c r="I1146" s="6" t="str">
         <f>VLOOKUP(F1146,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1147">
@@ -36530,7 +36530,7 @@
       </c>
       <c r="I1148" s="6" t="str">
         <f>VLOOKUP(F1148,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1149">
@@ -36592,7 +36592,7 @@
       </c>
       <c r="I1150" s="6" t="str">
         <f>VLOOKUP(F1150,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1151">
@@ -36654,7 +36654,7 @@
       </c>
       <c r="I1152" s="6" t="str">
         <f>VLOOKUP(F1152,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1153">
@@ -36716,7 +36716,7 @@
       </c>
       <c r="I1154" s="6" t="str">
         <f>VLOOKUP(F1154,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1155">
@@ -36809,7 +36809,7 @@
       </c>
       <c r="I1157" s="6" t="str">
         <f>VLOOKUP(F1157,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1158">
@@ -36902,7 +36902,7 @@
       </c>
       <c r="I1160" s="6" t="str">
         <f>VLOOKUP(F1160,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1161">
@@ -36995,7 +36995,7 @@
       </c>
       <c r="I1163" s="6" t="str">
         <f>VLOOKUP(F1163,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1164">
@@ -37088,7 +37088,7 @@
       </c>
       <c r="I1166" s="6" t="str">
         <f>VLOOKUP(F1166,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1167">
@@ -37212,7 +37212,7 @@
       </c>
       <c r="I1170" s="6" t="str">
         <f>VLOOKUP(F1170,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1171">
@@ -37336,7 +37336,7 @@
       </c>
       <c r="I1174" s="6" t="str">
         <f>VLOOKUP(F1174,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1175">
@@ -37429,7 +37429,7 @@
       </c>
       <c r="I1177" s="6" t="str">
         <f>VLOOKUP(F1177,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1178">
@@ -37491,7 +37491,7 @@
       </c>
       <c r="I1179" s="6" t="str">
         <f>VLOOKUP(F1179,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1180">
@@ -37615,7 +37615,7 @@
       </c>
       <c r="I1183" s="6" t="str">
         <f>VLOOKUP(F1183,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1184">
@@ -37739,7 +37739,7 @@
       </c>
       <c r="I1187" s="6" t="str">
         <f>VLOOKUP(F1187,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1188">
@@ -37832,7 +37832,7 @@
       </c>
       <c r="I1190" s="6" t="str">
         <f>VLOOKUP(F1190,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1191">
@@ -37925,7 +37925,7 @@
       </c>
       <c r="I1193" s="6" t="str">
         <f>VLOOKUP(F1193,lookups!$2:$110,3,FALSE)</f>
-        <v>Seagrass</v>
+        <v>Invasive seagrass</v>
       </c>
     </row>
     <row r="1194">
@@ -45396,216 +45396,216 @@
         <v>105</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C12" s="20" t="s">
         <v>109</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B15" s="20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B17" s="20" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B18" s="20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="20" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="20" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="20" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C27" s="20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>144</v>
+      </c>
+      <c r="C28" s="20" t="s">
         <v>142</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="20" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="30">
@@ -45616,7 +45616,7 @@
         <v>148</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="31">
@@ -45627,7 +45627,7 @@
         <v>150</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32">
@@ -45638,7 +45638,7 @@
         <v>152</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="33">
@@ -45649,7 +45649,7 @@
         <v>154</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34">
@@ -45660,7 +45660,7 @@
         <v>156</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35">
@@ -45671,7 +45671,7 @@
         <v>158</v>
       </c>
       <c r="C35" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="36">
@@ -45682,29 +45682,29 @@
         <v>160</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="B37" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="B37" s="20" t="s">
-        <v>163</v>
-      </c>
       <c r="C37" s="20" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B38" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="B38" s="20" t="s">
+      <c r="C38" s="20" t="s">
         <v>165</v>
-      </c>
-      <c r="C38" s="20" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="39">
@@ -45715,7 +45715,7 @@
         <v>167</v>
       </c>
       <c r="C39" s="20" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="40">
@@ -45726,7 +45726,7 @@
         <v>169</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="41">
@@ -45737,7 +45737,7 @@
         <v>171</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42">
@@ -45748,7 +45748,7 @@
         <v>173</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
     </row>
     <row r="43">

</xml_diff>